<commit_message>
fix(pricing): correct BW00-0 factory cost to exact 78.4615385 THB (FX 34.00) matching company source sheet
</commit_message>
<xml_diff>
--- a/docs/specs/BW00-0_pricing_comparison_sheet.xlsx
+++ b/docs/specs/BW00-0_pricing_comparison_sheet.xlsx
@@ -524,7 +524,7 @@
   <dimension ref="A1:W9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="128" customWidth="1" min="1" max="1"/>
+    <col width="111" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -559,7 +559,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>โครงสร้างรหัส: รหัสโมเดล [BW00] + จำนวนชิ้น [-0] + รหัสแพ็กเกจ [(P-BAG)] = BW00-0(P-BAG) | ค่าส่งเหมา 2,500 บ. เฉลี่ยในต้นทุน</t>
+          <t>อ้างอิงต้นทุนโรงงานจริง: US$2.31 (=15/6.5) x 34 บาท = 78.4615385 บาท | ค่าส่งเหมา 2,500 บ. เฉลี่ยในต้นทุน</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>฿83.08</t>
+          <t>฿78.46</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
@@ -744,7 +744,7 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>฿150.10</t>
+          <t>฿145.48</t>
         </is>
       </c>
       <c r="N5" s="8" t="inlineStr">
@@ -754,17 +754,17 @@
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
-          <t>฿99.90</t>
+          <t>฿104.52</t>
         </is>
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>฿4,995</t>
+          <t>฿5,226</t>
         </is>
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>41.8%</t>
         </is>
       </c>
       <c r="R5" s="8" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>฿38.90</t>
+          <t>฿43.52</t>
         </is>
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>฿1,945</t>
+          <t>฿2,176</t>
         </is>
       </c>
       <c r="U5" s="8" t="inlineStr">
         <is>
-          <t>20.6%</t>
+          <t>23.0%</t>
         </is>
       </c>
       <c r="V5" s="9" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>฿83.08</t>
+          <t>฿78.46</t>
         </is>
       </c>
       <c r="J6" s="11" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="M6" s="11" t="inlineStr">
         <is>
-          <t>฿125.10</t>
+          <t>฿120.48</t>
         </is>
       </c>
       <c r="N6" s="12" t="inlineStr">
@@ -871,17 +871,17 @@
       </c>
       <c r="O6" s="11" t="inlineStr">
         <is>
-          <t>฿104.90</t>
+          <t>฿109.52</t>
         </is>
       </c>
       <c r="P6" s="11" t="inlineStr">
         <is>
-          <t>฿10,490</t>
+          <t>฿10,952</t>
         </is>
       </c>
       <c r="Q6" s="12" t="inlineStr">
         <is>
-          <t>45.6%</t>
+          <t>47.6%</t>
         </is>
       </c>
       <c r="R6" s="12" t="inlineStr">
@@ -891,17 +891,17 @@
       </c>
       <c r="S6" s="11" t="inlineStr">
         <is>
-          <t>฿43.90</t>
+          <t>฿48.52</t>
         </is>
       </c>
       <c r="T6" s="11" t="inlineStr">
         <is>
-          <t>฿4,390</t>
+          <t>฿4,852</t>
         </is>
       </c>
       <c r="U6" s="12" t="inlineStr">
         <is>
-          <t>26.0%</t>
+          <t>28.7%</t>
         </is>
       </c>
       <c r="V6" s="9" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>฿83.08</t>
+          <t>฿78.46</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
@@ -978,7 +978,7 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>฿108.43</t>
+          <t>฿103.81</t>
         </is>
       </c>
       <c r="N7" s="8" t="inlineStr">
@@ -988,17 +988,17 @@
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
-          <t>฿106.57</t>
+          <t>฿111.19</t>
         </is>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>฿31,971</t>
+          <t>฿33,356</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>49.6%</t>
+          <t>51.7%</t>
         </is>
       </c>
       <c r="R7" s="8" t="inlineStr">
@@ -1008,17 +1008,17 @@
       </c>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>฿40.57</t>
+          <t>฿45.19</t>
         </is>
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>฿12,171</t>
+          <t>฿13,556</t>
         </is>
       </c>
       <c r="U7" s="8" t="inlineStr">
         <is>
-          <t>27.2%</t>
+          <t>30.3%</t>
         </is>
       </c>
       <c r="V7" s="9" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>฿83.08</t>
+          <t>฿78.46</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="M8" s="11" t="inlineStr">
         <is>
-          <t>฿105.10</t>
+          <t>฿100.48</t>
         </is>
       </c>
       <c r="N8" s="12" t="inlineStr">
@@ -1105,17 +1105,17 @@
       </c>
       <c r="O8" s="11" t="inlineStr">
         <is>
-          <t>฿94.90</t>
+          <t>฿99.52</t>
         </is>
       </c>
       <c r="P8" s="11" t="inlineStr">
         <is>
-          <t>฿47,452</t>
+          <t>฿49,759</t>
         </is>
       </c>
       <c r="Q8" s="12" t="inlineStr">
         <is>
-          <t>47.5%</t>
+          <t>49.8%</t>
         </is>
       </c>
       <c r="R8" s="12" t="inlineStr">
@@ -1125,17 +1125,17 @@
       </c>
       <c r="S8" s="11" t="inlineStr">
         <is>
-          <t>฿33.90</t>
+          <t>฿38.52</t>
         </is>
       </c>
       <c r="T8" s="11" t="inlineStr">
         <is>
-          <t>฿16,952</t>
+          <t>฿19,259</t>
         </is>
       </c>
       <c r="U8" s="12" t="inlineStr">
         <is>
-          <t>24.4%</t>
+          <t>27.7%</t>
         </is>
       </c>
       <c r="V8" s="9" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>฿83.08</t>
+          <t>฿78.46</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>฿102.60</t>
+          <t>฿97.98</t>
         </is>
       </c>
       <c r="N9" s="8" t="inlineStr">
@@ -1222,17 +1222,17 @@
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>฿82.40</t>
+          <t>฿87.02</t>
         </is>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>฿82,403</t>
+          <t>฿87,018</t>
         </is>
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>44.5%</t>
+          <t>47.0%</t>
         </is>
       </c>
       <c r="R9" s="8" t="inlineStr">
@@ -1242,17 +1242,17 @@
       </c>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>฿26.40</t>
+          <t>฿31.02</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>฿26,403</t>
+          <t>฿31,018</t>
         </is>
       </c>
       <c r="U9" s="8" t="inlineStr">
         <is>
-          <t>20.5%</t>
+          <t>24.0%</t>
         </is>
       </c>
       <c r="V9" s="9" t="inlineStr">
@@ -1280,7 +1280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="74" customWidth="1" min="1" max="1"/>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>EXW $2.31 USD (Vacuum cup in simple dark blue gift bag)</t>
+          <t>EXW US$2.31 (Vacuum cup in simple dark blue gift bag)</t>
         </is>
       </c>
     </row>
@@ -1367,168 +1367,219 @@
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>ความจุ</t>
+          <t>ต้นทุนโรงงานจริง (USD)</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>450 ml</t>
+          <t>US$ 2.31 (=15/6.5)</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>ขนาดกระชับมือ พกพาสะดวก</t>
+          <t>อ้างอิงตรงจาก Row 5846 ในไฟล์ต้นทุน 01-ต้นทุน-20260612</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>ขนาดสินค้า</t>
+          <t>อัตราแลกเปลี่ยน</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>เส้นผ่านศูนย์กลาง 65 มม. x สูง 230 มม.</t>
+          <t>34.00 บาท / USD</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>น้ำหนักประมาณ 320 กรัม</t>
+          <t>อัตราที่ใช้ในคอลัมน์ 'บาท' ของไฟล์ต้นทุนบริษัท</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="inlineStr">
         <is>
-          <t>วัสดุตัวแก้ว</t>
+          <t>ต้นทุนโรงงานจริง (บาท)</t>
         </is>
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>สแตนเลส SUS304 Food Grade สองชั้นสูญญากาศ</t>
+          <t>78.4615385 บาท (78.46 ฿)</t>
         </is>
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>ปลอดภัย ไร้สนิม ไร้สาร BPA</t>
+          <t>ตรงกับเซลล์ในคอลัมน์ 'บาท' 100%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>ฟังก์ชันฝาปิด</t>
+          <t>ความจุ</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Touch Sensor LED Temperature Display</t>
+          <t>450 ml</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>แตะฝาเพื่อดูอุณหภูมิเครื่องดื่มแบบเรียลไทม์ พร้อมซีลซิลิโคนกันรั่วซึม</t>
+          <t>ขนาดกระชับมือ พกพาสะดวก</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>ประสิทธิภาพการเก็บอุณหภูมิ</t>
+          <t>ขนาดสินค้า</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>เก็บความร้อน 6 - 12 ชม. / เก็บความเย็น 12 - 24 ชม.</t>
+          <t>เส้นผ่านศูนย์กลาง 65 มม. x สูง 230 มม.</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>ทดสอบตามมาตรฐานสากล</t>
+          <t>น้ำหนักประมาณ 320 กรัม</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>สีที่มีให้เลือก (8 สี)</t>
+          <t>วัสดุตัวแก้ว</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>น้ำเงิน, เงิน, ดำ, แดง, ทอง, ชมพู, ส้ม, ฟ้าอ่อน</t>
+          <t>สแตนเลส SUS304 Food Grade สองชั้นสูญญากาศ</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>สกรีนโลโก้หรือเลเซอร์ได้ทุกสี</t>
+          <t>ปลอดภัย ไร้สนิม ไร้สาร BPA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>ตัวเลือกแพ็กเกจ 1</t>
+          <t>ฟังก์ชันฝาปิด</t>
         </is>
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>(P-BAG) ถุงของขวัญ Dark Blue Gift Bag หูหิ้ว</t>
+          <t>Touch Sensor LED Temperature Display</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>รวมอยู่ในราคามาตรฐานแล้ว (ฟรี)</t>
+          <t>แตะฝาเพื่อดูอุณหภูมิเครื่องดื่มแบบเรียลไทม์ พร้อมซีลซิลิโคนกันรั่วซึม</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>ตัวเลือกแพ็กเกจ 2</t>
+          <t>ประสิทธิภาพการเก็บอุณหภูมิ</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>(P-01) กล่องของขวัญเดี่ยวแบบแข็งเปิดฝาบน ฟองน้ำ EVA</t>
+          <t>เก็บความร้อน 6 - 12 ชม. / เก็บความเย็น 12 - 24 ชม.</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>เพิ่ม 25.00 บาท/ชุด</t>
+          <t>ทดสอบตามมาตรฐานสากล</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>ตัวเลือกแพ็กเกจ 3</t>
+          <t>สีที่มีให้เลือก (8 สี)</t>
         </is>
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>(P-TUBE) กระบอกของขวัญทรงกลมพรีเมียม ปั๊มฟอยล์</t>
+          <t>น้ำเงิน, เงิน, ดำ, แดง, ทอง, ชมพู, ส้ม, ฟ้าอ่อน</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>เพิ่ม 20.00 บาท/ชุด</t>
+          <t>สกรีนโลโก้หรือเลเซอร์ได้ทุกสี</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
+          <t>ตัวเลือกแพ็กเกจ 1</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>(P-BAG) ถุงของขวัญ Dark Blue Gift Bag หูหิ้ว</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>รวมอยู่ในราคามาตรฐานแล้ว (ฟรี)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>ตัวเลือกแพ็กเกจ 2</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>(P-01) กล่องของขวัญเดี่ยวแบบแข็งเปิดฝาบน ฟองน้ำ EVA</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>เพิ่ม 25.00 บาท/ชุด</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>ตัวเลือกแพ็กเกจ 3</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>(P-TUBE) กระบอกของขวัญทรงกลมพรีเมียม ปั๊มฟอยล์</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>เพิ่ม 20.00 บาท/ชุด</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
           <t>การจัดส่ง (Direct Single Drop)</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>ท่าเรือคลองเตย/แหลมฉบัง -&gt; จุดหมายลูกค้า 1 จุด</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>ค่ารถเหมา 2,500 บาท เฉลี่ยในต้นทุน ออกใบเสนอราคาฟรีค่าส่ง</t>
         </is>

</xml_diff>